<commit_message>
feat: implement application scaffolding including UI controllers, data repositories, and solver orchestration logic
</commit_message>
<xml_diff>
--- a/data/files/input_data.xlsx
+++ b/data/files/input_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ludov\Documents\Esercizi programmazione\Python\Progetto Dashboard gestionale\data\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63AF4A37-192F-46F3-879C-79333D2C8202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6468B44-6E91-44C3-A943-466C5D1EEF57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attività e Risorse" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="41">
   <si>
     <t>Durata Minima</t>
   </si>
@@ -163,9 +163,6 @@
   <si>
     <t>ID Attività</t>
   </si>
-  <si>
-    <t>30-31</t>
-  </si>
 </sst>
 </file>
 
@@ -214,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -240,15 +237,50 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <protection locked="0" hidden="0"/>
@@ -300,45 +332,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -353,13 +346,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5AB97735-4C45-4F45-954D-45D0C1CF41B2}" name="Tabella1" displayName="Tabella1" ref="A1:Q600" totalsRowShown="0" headerRowDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5AB97735-4C45-4F45-954D-45D0C1CF41B2}" name="Tabella1" displayName="Tabella1" ref="A1:Q600" totalsRowShown="0" headerRowDxfId="16">
   <autoFilter ref="A1:Q600" xr:uid="{5AB97735-4C45-4F45-954D-45D0C1CF41B2}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{140F7A0F-0B8D-4546-AD97-2DBBA7C8EE15}" name="ID Attività" dataDxfId="8">
+    <tableColumn id="1" xr3:uid="{140F7A0F-0B8D-4546-AD97-2DBBA7C8EE15}" name="ID Attività" dataDxfId="15">
       <calculatedColumnFormula>IF(B2&lt;&gt;"",COUNTA($B2:B$3),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{29D82F95-D176-4FA3-920E-CECEC04024C8}" name="Nome Attività" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{29D82F95-D176-4FA3-920E-CECEC04024C8}" name="Nome Attività" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{9C5178DF-D2C9-4847-8482-CFC6217B40C3}" name="Durata Minima"/>
     <tableColumn id="4" xr3:uid="{5F50A607-E9F7-43F2-AC3E-D7681021E4E1}" name="Durata Massima (Opzionale)"/>
     <tableColumn id="5" xr3:uid="{39A771DA-D40D-4B99-B294-B041353A9E10}" name="Risorsa 1"/>
@@ -381,33 +374,33 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6D529CD1-6F47-428F-8F81-5496EB0CC66F}" name="Tabella2" displayName="Tabella2" ref="A1:F600" totalsRowShown="0" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6D529CD1-6F47-428F-8F81-5496EB0CC66F}" name="Tabella2" displayName="Tabella2" ref="A1:F600" totalsRowShown="0" dataDxfId="13">
   <autoFilter ref="A1:F600" xr:uid="{6D529CD1-6F47-428F-8F81-5496EB0CC66F}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{EE66BBF7-C291-4B31-BD9A-04ACE2CE45BD}" name="ID Attività" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{EE66BBF7-C291-4B31-BD9A-04ACE2CE45BD}" name="ID Attività" dataDxfId="12">
       <calculatedColumnFormula>IF('Attività e Risorse'!A3&lt;&gt;"",'Attività e Risorse'!A3,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2546B960-92C5-49E2-8D27-0243D21C1E6B}" name="Nome Attività" dataDxfId="4">
+    <tableColumn id="2" xr3:uid="{2546B960-92C5-49E2-8D27-0243D21C1E6B}" name="Nome Attività" dataDxfId="11">
       <calculatedColumnFormula>IF('Attività e Risorse'!B3&lt;&gt;"",'Attività e Risorse'!B3,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{42465140-EC98-4E8C-82C0-DB27335FDC45}" name="Data di Rilascio Minima" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{92DE7C69-76EB-4556-9209-F9AAF450C00E}" name="Data di Rilascio Massima" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{760EA89A-1124-461E-BE59-007002487457}" name="Data di Scadenza Minima" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{6C8C3130-BDF8-49EE-8827-482B59DDBE03}" name="Data di Scadenza Massima" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{42465140-EC98-4E8C-82C0-DB27335FDC45}" name="Data di Rilascio Minima" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{92DE7C69-76EB-4556-9209-F9AAF450C00E}" name="Data di Rilascio Massima" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{760EA89A-1124-461E-BE59-007002487457}" name="Data di Scadenza Minima" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{6C8C3130-BDF8-49EE-8827-482B59DDBE03}" name="Data di Scadenza Massima" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3482686D-62FF-4551-A672-CB8416B52BCF}" name="Tabella4" displayName="Tabella4" ref="A1:E600" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3482686D-62FF-4551-A672-CB8416B52BCF}" name="Tabella4" displayName="Tabella4" ref="A1:E600" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <autoFilter ref="A1:E600" xr:uid="{3482686D-62FF-4551-A672-CB8416B52BCF}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7008AD5F-8180-4198-A523-CCDEB7BEEFDE}" name="Attività Precedente" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{9726E98F-48CF-4471-9C2D-A346E5D86FDB}" name="Attività Successiva" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{2CFF0289-F7AA-4345-B6E6-8A98A5E6F650}" name="Tipo di Legame" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{1AB52DD9-E9FB-4570-B1B8-66A5F8F7ED05}" name="Distanza Minima (Lag temporale)" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{11993FDA-6845-43B1-9523-15AC1D431AB6}" name="Distanza Massima (Opzionale)" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{7008AD5F-8180-4198-A523-CCDEB7BEEFDE}" name="Attività Precedente" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{9726E98F-48CF-4471-9C2D-A346E5D86FDB}" name="Attività Successiva" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{2CFF0289-F7AA-4345-B6E6-8A98A5E6F650}" name="Tipo di Legame" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{1AB52DD9-E9FB-4570-B1B8-66A5F8F7ED05}" name="Distanza Minima (Lag temporale)" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{11993FDA-6845-43B1-9523-15AC1D431AB6}" name="Distanza Massima (Opzionale)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -792,13 +785,13 @@
       <c r="BG1" s="8"/>
     </row>
     <row r="2" spans="1:59" s="2" customFormat="1" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="E2" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="F2" s="9">
+      <c r="E2" s="8">
+        <v>30</v>
+      </c>
+      <c r="F2" s="8">
         <v>20</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="8">
         <v>15</v>
       </c>
       <c r="H2" s="8"/>
@@ -887,9 +880,7 @@
       <c r="C5" s="6">
         <v>4</v>
       </c>
-      <c r="D5" s="6">
-        <v>8</v>
-      </c>
+      <c r="D5" s="6"/>
       <c r="E5" s="6">
         <v>4</v>
       </c>
@@ -1017,9 +1008,7 @@
       <c r="C9" s="6">
         <v>3</v>
       </c>
-      <c r="D9" s="6">
-        <v>7</v>
-      </c>
+      <c r="D9" s="6"/>
       <c r="E9" s="6">
         <v>6</v>
       </c>
@@ -1115,9 +1104,7 @@
       <c r="C12" s="6">
         <v>12</v>
       </c>
-      <c r="D12" s="6">
-        <v>14</v>
-      </c>
+      <c r="D12" s="6"/>
       <c r="E12" s="6">
         <v>1</v>
       </c>
@@ -14145,9 +14132,7 @@
       <c r="C3" s="7">
         <v>46157</v>
       </c>
-      <c r="D3" s="7">
-        <v>46159</v>
-      </c>
+      <c r="D3" s="7"/>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
     </row>
@@ -14207,9 +14192,7 @@
       <c r="E7" s="7">
         <v>46183</v>
       </c>
-      <c r="F7" s="7">
-        <v>46185</v>
-      </c>
+      <c r="F7" s="7"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8">

</xml_diff>